<commit_message>
Make Where's my parcel FAQ only: answers end the chat
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NH7tHcFV3YFRTo4Z6ab4aP
</commit_message>
<xml_diff>
--- a/Ninja_Bot_v2_Flow_Logic.xlsx
+++ b/Ninja_Bot_v2_Flow_Logic.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Bot Copy'!$A$4:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Issue Trend (L1)'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Future Updates'!$A$4:$J$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Change Log'!$A$4:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Change Log'!$A$4:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Developer Prompt'!$A$4:$A$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D33"/>
+  <dimension ref="B2:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -906,23 +906,31 @@
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Values in [brackets] are filled from a tool at run time. "TO CONFIRM" marks an open decision.</t>
+          <t>Where's my parcel (flow A) is FAQ only: the answer screens A2 to A6 end the chat, with no button and no follow-up question.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="B33" s="14" t="inlineStr">
         <is>
+          <t>Values in [brackets] are filled from a tool at run time. "TO CONFIRM" marks an open decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
           <t>Interactive map: https://claude.ai/artifact/Qa1K4HqDpn8CzZYuwhbxzk · Simulator: https://claude.ai/artifact/RmwMNJN5bK15PSEcVGDCFe</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="B33:D33"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B34:D34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -934,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1019,8 +1027,36 @@
       </c>
       <c r="F5" s="18" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Flow Mapping, Routing Logic, Issue Coverage</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>A2–A6, R09–R13</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Where's my parcel changed to FAQ only: answers end the chat, no Did this help?, no agent or case buttons.</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F5"/>
+  <autoFilter ref="A4:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1066,9 +1102,10 @@
 2. Read Routing Logic: implement every rule in order. Rules are the only place branching is decided. Do not hard-code branches in screens.
 3. Read Integrations: build a thin client per INT ID. Fields marked TO CONFIRM need Tech to confirm before release.
 4. Read Data Fields: keep the session object with those fields and send the "Passed to agent = Yes" fields in the handoff payload.
-5. Global rules: Main menu and Talk to an agent on every screen except handoff and global screens. Never show POD, receiver name, signature or full address in the bot.
-6. Values in [brackets] come from a tool or from INT10 config. Do not hard-code them.
-7. Log the path and CSAT (INT09). Acceptance: every issue type in Issue Coverage can be reached in three taps or fewer after the tracking ID, and every escalation carries tracking ID, parcel status, flow, auto-tag, priority, identity-check flag and remarks.</t>
+5. Where's my parcel (A2 to A6) is FAQ only: after the answer, end the chat. No buttons, no question.
+6. Global rules: Main menu and Talk to an agent on every screen except handoff and global screens. Never show POD, receiver name, signature or full address in the bot.
+7. Values in [brackets] come from a tool or from INT10 config. Do not hard-code them.
+8. Log the path and CSAT (INT09). Acceptance: every issue type in Issue Coverage can be reached in three taps or fewer after the tracking ID, and every escalation carries tracking ID, parcel status, flow, auto-tag, priority, identity-check flag and remarks.</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1269,12 @@
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Self-serve</t>
+          <t>Self-serve (FAQ)</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr">
         <is>
-          <t>Status shown automatically after tracking ID</t>
+          <t>Status shown automatically after tracking ID, chat ends</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1351,12 @@
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Self-serve</t>
+          <t>Self-serve (FAQ)</t>
         </is>
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>ETA shown, no agent needed</t>
+          <t>ETA shown, chat ends</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1597,12 @@
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>Escalate (case)</t>
+          <t>Self-serve (FAQ)</t>
         </is>
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>Apologise, flag to team</t>
+          <t>FAQ answer, chat ends. No case is created</t>
         </is>
       </c>
     </row>
@@ -1760,17 +1797,17 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>A6 → H1</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Escalate (agent)</t>
+          <t>Self-serve (FAQ)</t>
         </is>
       </c>
       <c r="I19" s="18" t="inlineStr">
         <is>
-          <t>Show reason, agent fixes address / special instruction</t>
+          <t>FAQ answer with the reason, chat ends</t>
         </is>
       </c>
     </row>
@@ -1929,12 +1966,12 @@
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>Escalate (agent)</t>
+          <t>Self-serve (FAQ)</t>
         </is>
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>Shown as On hold / returning; cannot revert self-serve</t>
+          <t>Shown as On hold / returning, chat ends</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2585,7 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Info (FAQ)</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
@@ -2563,21 +2600,13 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Did this help? Yes | No</t>
-        </is>
-      </c>
-      <c r="G11" s="18" t="inlineStr">
-        <is>
-          <t>Next → G1 (Did this help?)
-No → Talk to an agent → H1 (Talk to an agent)
-Change details → D2 (Change address / phone)
-Update special instruction → D3 (Note for courier)
-Main menu → W1 (Main menu)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr"/>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>INT01, INT08</t>
+          <t>INT01</t>
         </is>
       </c>
       <c r="I11" s="18" t="inlineStr">
@@ -2587,7 +2616,7 @@
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
-          <t>Self-serve</t>
+          <t>FAQ, ends here</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -2614,7 +2643,7 @@
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>Info + Escalate</t>
+          <t>Info (FAQ)</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -2624,23 +2653,18 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>Sorry, your parcel is taking longer than expected. Last update: [Last scan]. We'll flag this to our team to check it for you.</t>
+          <t>Sorry, your parcel is taking longer than expected. Last update: [Last scan]. Delays like this are usually resolved within a few days.</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Flag it to the team | Talk to an agent</t>
-        </is>
-      </c>
-      <c r="G12" s="18" t="inlineStr">
-        <is>
-          <t>Next → H2 (Case created)
-Talk to an agent → H1 (Talk to an agent)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr"/>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>INT10, INT05</t>
+          <t>INT10</t>
         </is>
       </c>
       <c r="I12" s="18" t="inlineStr">
@@ -2650,7 +2674,7 @@
       </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
-          <t>Escalate (case)</t>
+          <t>FAQ, ends here</t>
         </is>
       </c>
       <c r="K12" s="18" t="inlineStr">
@@ -2677,7 +2701,7 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Info (FAQ)</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
@@ -2692,25 +2716,19 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Leave a note for the courier | Change my delivery | Main menu</t>
-        </is>
-      </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>Note for courier → D3 (Note for courier)
-Change options → D1 (Change options)
-Main menu → W1 (Main menu)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr"/>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>INT08</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I13" s="18" t="inlineStr"/>
       <c r="J13" s="18" t="inlineStr">
         <is>
-          <t>Self-serve</t>
+          <t>FAQ, ends here</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -2737,7 +2755,7 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Info (FAQ)</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
@@ -2752,16 +2770,10 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Main menu | Talk to an agent</t>
-        </is>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
-        <is>
-          <t>Next → G1 (Did this help?)
-Main menu → W1 (Main menu)
-Talk to an agent → H1 (Talk to an agent)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr">
         <is>
           <t>INT01</t>
@@ -2774,7 +2786,7 @@
       </c>
       <c r="J14" s="18" t="inlineStr">
         <is>
-          <t>Self-serve</t>
+          <t>FAQ, ends here</t>
         </is>
       </c>
       <c r="K14" s="18" t="inlineStr">
@@ -2801,7 +2813,7 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Info (FAQ)</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
@@ -2811,23 +2823,18 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Your parcel is currently [On hold / Returning to seller]. Reason: [General reason, e.g. we need more address details].</t>
+          <t>Your parcel is currently [On hold / Returning to seller]. Reason: [General reason, e.g. we need more address details]. Once the issue is fixed, your parcel will move again.</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Talk to an agent | Main menu</t>
-        </is>
-      </c>
-      <c r="G15" s="18" t="inlineStr">
-        <is>
-          <t>Next → H1 (Talk to an agent)
-Main menu → W1 (Main menu)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr"/>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>INT01, INT06</t>
+          <t>INT01</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr">
@@ -2837,7 +2844,7 @@
       </c>
       <c r="J15" s="18" t="inlineStr">
         <is>
-          <t>Escalate</t>
+          <t>FAQ, ends here</t>
         </is>
       </c>
       <c r="K15" s="18" t="inlineStr">
@@ -5788,7 +5795,7 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A2 (FAQ answer, chat ends)</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
@@ -5803,7 +5810,7 @@
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J13" s="18" t="inlineStr">
@@ -5841,12 +5848,12 @@
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>INT01</t>
+          <t>INT01, INT10</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A3 (FAQ answer, chat ends)</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
@@ -5861,7 +5868,7 @@
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J14" s="18" t="inlineStr">
@@ -5908,7 +5915,7 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A4 (FAQ answer, chat ends)</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
@@ -5962,7 +5969,7 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A5 (FAQ answer, chat ends)</t>
         </is>
       </c>
       <c r="G16" s="18" t="inlineStr">
@@ -5977,7 +5984,7 @@
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J16" s="18" t="inlineStr">
@@ -6020,7 +6027,7 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>A6 (FAQ answer, chat ends)</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
@@ -6035,7 +6042,7 @@
       </c>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J17" s="18" t="inlineStr">
@@ -6045,7 +6052,7 @@
       </c>
       <c r="K17" s="18" t="inlineStr">
         <is>
-          <t>Show general reason only</t>
+          <t>Show general reason only. FAQ only: no agent button, no question after the answer</t>
         </is>
       </c>
       <c r="L17" s="33" t="inlineStr">
@@ -7601,7 +7608,7 @@
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>H2, B3, B5, C3, ED, A3, E5</t>
+          <t>H2, B3, B5, C3, ED, E5</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
@@ -7648,7 +7655,7 @@
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>H1, HC, D2, D5, D9, A6, T2</t>
+          <t>H1, HC, D2, D5, D9, T2</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
@@ -7742,7 +7749,7 @@
       </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>A2, A4, D10</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
@@ -8170,7 +8177,7 @@
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>R10, R17, R18, R28, R29</t>
+          <t>R17, R18, R28, R29</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -8841,7 +8848,7 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Did this help? Yes | No</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F11" s="33" t="inlineStr"/>
@@ -8870,12 +8877,12 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Sorry, your parcel is taking longer than expected. Last update: [Last scan]. We'll flag this to our team to check it for you.</t>
+          <t>Sorry, your parcel is taking longer than expected. Last update: [Last scan]. Delays like this are usually resolved within a few days.</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>Flag it to the team | Talk to an agent</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" s="33" t="inlineStr"/>
@@ -8909,7 +8916,7 @@
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Leave a note for the courier | Change my delivery | Main menu</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F13" s="33" t="inlineStr"/>
@@ -8943,7 +8950,7 @@
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>Main menu | Talk to an agent</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F14" s="33" t="inlineStr"/>
@@ -8972,12 +8979,12 @@
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>Your parcel is currently [On hold / Returning to seller]. Reason: [General reason, e.g. we need more address details].</t>
+          <t>Your parcel is currently [On hold / Returning to seller]. Reason: [General reason, e.g. we need more address details]. Once the issue is fixed, your parcel will move again.</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Talk to an agent | Main menu</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F15" s="33" t="inlineStr"/>

</xml_diff>

<commit_message>
Split change options into address, contact number, and both
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NH7tHcFV3YFRTo4Z6ab4aP
</commit_message>
<xml_diff>
--- a/Ninja_Bot_v2_Flow_Logic.xlsx
+++ b/Ninja_Bot_v2_Flow_Logic.xlsx
@@ -3376,12 +3376,12 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Address or phone | Map pin location | Note for courier | Delivery date | Collect at pickup point | Deliver to my door instead | Keep at pickup point longer | Cancel delivery</t>
+          <t>Address | Contact number | Address and contact number | Map pin location | Note for courier | Delivery date | Collect at pickup point | Deliver to my door instead | Keep at pickup point longer | Cancel delivery</t>
         </is>
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Address or phone → D2 (Change address / phone)
+          <t>Address / contact / both → D2 (Change address / contact number)
 Map pin → D9 (Map pin)
 Note for courier → D3 (Note for courier)
 Delivery date → D4 (Pick delivery date)
@@ -3427,12 +3427,12 @@
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Change address / phone</t>
+          <t>Change address / contact number</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
         <is>
-          <t>For your security, changes to the delivery address or phone number are made by our agent after a quick identity check.</t>
+          <t>For your security, changes to the delivery address, contact number or both are made by our agent after a quick identity check.</t>
         </is>
       </c>
       <c r="F25" s="18" t="inlineStr">
@@ -3753,7 +3753,7 @@
       <c r="G30" s="18" t="inlineStr">
         <is>
           <t>Confirm → D10 (Change saved)
-Change address / phone → D2 (Change address / phone)</t>
+Change address / phone → D2 (Change address / contact number)</t>
         </is>
       </c>
       <c r="H30" s="18" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Customer asks to change address / phone, pickup point or map pin</t>
+          <t>Customer asks to change address, contact number (or both), pickup point or map pin</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="E24" s="18" t="inlineStr">
         <is>
-          <t>Address or phone | Map pin location | Note for courier | Delivery date | Collect at pickup point | Deliver to my door instead | Keep at pickup point longer | Cancel delivery</t>
+          <t>Address | Contact number | Address and contact number | Map pin location | Note for courier | Delivery date | Collect at pickup point | Deliver to my door instead | Keep at pickup point longer | Cancel delivery</t>
         </is>
       </c>
       <c r="F24" s="33" t="inlineStr"/>
@@ -9314,12 +9314,12 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Change address / phone</t>
+          <t>Change address / contact number</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>For your security, changes to the delivery address or phone number are made by our agent after a quick identity check.</t>
+          <t>For your security, changes to the delivery address, contact number or both are made by our agent after a quick identity check.</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">

</xml_diff>